<commit_message>
feat: add streamlit web ui for parser
- Create interactive web interface using Streamlit
- Add 5-tab workflow: Connection, Upload, Configure, Run, Results
- Real-time progress tracking during parsing
- File upload and preview with validation
- Dry-run mode for safe testing
- Detailed logging and result download
- Auto-detect PAT authentication
- Configuration from settings.json
- Setup scripts for Windows and Linux/macOS
- Comprehensive documentation and quick start guide
</commit_message>
<xml_diff>
--- a/UV-Sheets_protocol.xlsx
+++ b/UV-Sheets_protocol.xlsx
@@ -530,7 +530,7 @@
       <c r="J2" t="n">
         <v>10</v>
       </c>
-      <c r="K2" t="b">
+      <c r="K2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="J6" t="n">
         <v>5</v>
       </c>
-      <c r="K6" t="b">
+      <c r="K6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -713,7 +713,7 @@
       <c r="J7" t="n">
         <v>6</v>
       </c>
-      <c r="K7" t="b">
+      <c r="K7" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>